<commit_message>
add missing reference products
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-Carma-CCS.xlsx
+++ b/premise/data/additional_inventories/lci-Carma-CCS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romain/GitHub/premise/premise/data/additional_inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E191EE4-9E96-A446-8FF5-AF329E15E435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E5E7A8-6010-9048-AF0E-1A687DC2E85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="760" windowWidth="25800" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43600" yWindow="240" windowWidth="25800" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Carma CCS" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14704" uniqueCount="842">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14705" uniqueCount="843">
   <si>
     <t>Database</t>
   </si>
@@ -2562,6 +2562,9 @@
   </si>
   <si>
     <t>market for nickel, 99.5%</t>
+  </si>
+  <si>
+    <t>sand</t>
   </si>
 </sst>
 </file>
@@ -69801,6 +69804,9 @@
       <c r="K2568" t="s">
         <v>57</v>
       </c>
+      <c r="L2568" t="s">
+        <v>842</v>
+      </c>
     </row>
     <row r="2569" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2569" t="s">

</xml_diff>